<commit_message>
DNN-Based Model Tuning feature refactored.
</commit_message>
<xml_diff>
--- a/reports/HW-Chars.Recognition.Site/models.eval-results.xlsx
+++ b/reports/HW-Chars.Recognition.Site/models.eval-results.xlsx
@@ -27,9 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>Model</t>
+  </si>
+  <si>
+    <t>Hidden Layers</t>
   </si>
   <si>
     <t>Accuracy</t>
@@ -53,16 +56,10 @@
     <t>DNN-Based-Basic MCC</t>
   </si>
   <si>
-    <t>0.898489236831665</t>
-  </si>
-  <si>
     <t>+</t>
   </si>
   <si>
-    <t>Tuned DNN MCC Final</t>
-  </si>
-  <si>
-    <t>0.872517168521881</t>
+    <t>Tuned DNN MCC Final:</t>
   </si>
   <si>
     <t>CNN-Based-Basic MCC</t>
@@ -698,7 +695,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -708,14 +705,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1242,71 +1233,89 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="4"/>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="21.4545454545455" customWidth="1"/>
-    <col min="2" max="2" width="19.1818181818182" customWidth="1"/>
-    <col min="4" max="4" width="8.72727272727273" style="2"/>
+    <col min="2" max="3" width="12.8181818181818" customWidth="1"/>
+    <col min="5" max="5" width="8.72727272727273" style="2"/>
+    <col min="7" max="7" width="12.8181818181818"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:5">
-      <c r="A1" s="3" t="s">
+    <row r="1" s="1" customFormat="1" spans="1:6">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="5" t="s">
         <v>8</v>
       </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
       <c r="C4">
+        <v>0.897526204586029</v>
+      </c>
+      <c r="D4">
         <v>0.319</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>0.906163454055786</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>0.906584799289703</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
+    <row r="33" spans="1:1">
+      <c r="A33" t="s">
         <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>